<commit_message>
limiting the report generation for all results
</commit_message>
<xml_diff>
--- a/api/templates/all_results/en.xlsx
+++ b/api/templates/all_results/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24701"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\ubuntu\aspect\api\templates\export\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\ubuntu\aspect\api\templates\all_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96FEE4F7-E4C7-43CA-9646-339CBC5929C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B201FB5-DBEA-425D-AE05-0F6EE12A111A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21220" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -130,9 +130,6 @@
     <t>&lt;Table&gt;</t>
   </si>
   <si>
-    <t>Printed on &lt;date&gt;</t>
-  </si>
-  <si>
     <t>Aspect Results</t>
   </si>
   <si>
@@ -203,6 +200,9 @@
   </si>
   <si>
     <t>&lt;errorCode&gt;</t>
+  </si>
+  <si>
+    <t>Printed on &lt;Dates&gt;</t>
   </si>
 </sst>
 </file>
@@ -863,12 +863,12 @@
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8"/>
@@ -903,46 +903,46 @@
     </row>
     <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C5" s="19"/>
       <c r="D5" s="19"/>
       <c r="E5" s="19"/>
       <c r="F5" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="G5" s="21" t="s">
-        <v>48</v>
-      </c>
       <c r="H5" s="21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I5" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="J5" s="21" t="s">
-        <v>52</v>
-      </c>
       <c r="K5" s="18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19"/>
       <c r="B6" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="15" t="s">
-        <v>38</v>
-      </c>
       <c r="D6" s="15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F6" s="22"/>
       <c r="G6" s="22"/>
@@ -953,37 +953,37 @@
     </row>
     <row r="7" spans="1:11" s="2" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>42</v>
-      </c>
       <c r="E7" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I7" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="J7" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="J7" s="17" t="s">
-        <v>54</v>
-      </c>
       <c r="K7" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Extracted Device column from Ssample Collection Site column in all results report
</commit_message>
<xml_diff>
--- a/api/templates/all_results/en.xlsx
+++ b/api/templates/all_results/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24701"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\ubuntu\aspect\api\templates\all_results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\all_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F6B89A-9786-4A8E-A7AA-8CCDC0C77FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F9EBA44-F8B5-46DF-9F2A-40A28D26D09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5340" yWindow="5340" windowWidth="28800" windowHeight="15410" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -287,7 +287,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -336,6 +336,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -383,7 +420,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -434,6 +471,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="43" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -452,54 +492,66 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="43" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="44">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="3" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="5" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="7" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="9" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="11" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="13" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="15" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="17" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="19" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="21" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="23" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="25" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="27" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="29" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="31" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="33" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="35" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="37" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="39" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="41" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="6" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="8" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="10" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="12" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="14" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="16" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="18" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="20" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="22" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="24" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="26" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="28" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="30" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="32" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="34" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="36" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="38" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="40" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="42" builtinId="9" hidden="1"/>
-    <cellStyle name="Incorrecto" xfId="43" builtinId="27"/>
+    <cellStyle name="Bad" xfId="43" builtinId="27"/>
+    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="24" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="26" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="28" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="23" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="25" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="27" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
@@ -866,27 +918,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.5" style="5" customWidth="1"/>
-    <col min="2" max="2" width="23.08203125" style="7" customWidth="1"/>
-    <col min="3" max="3" width="22.4140625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="23.09765625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="22.3984375" style="8" customWidth="1"/>
     <col min="4" max="4" width="18.5" style="8" customWidth="1"/>
-    <col min="5" max="5" width="28.58203125" style="9" customWidth="1"/>
-    <col min="6" max="6" width="21.4140625" style="9" customWidth="1"/>
-    <col min="7" max="7" width="21.33203125" style="9" customWidth="1"/>
-    <col min="8" max="8" width="11.9140625" style="9" customWidth="1"/>
-    <col min="9" max="9" width="17.1640625" style="9" customWidth="1"/>
-    <col min="10" max="10" width="15.9140625" style="9" customWidth="1"/>
-    <col min="11" max="11" width="20.6640625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="28.59765625" style="9" customWidth="1"/>
+    <col min="6" max="6" width="21.3984375" style="9" customWidth="1"/>
+    <col min="7" max="7" width="21.296875" style="9" customWidth="1"/>
+    <col min="8" max="8" width="11.8984375" style="9" customWidth="1"/>
+    <col min="9" max="9" width="17.19921875" style="9" customWidth="1"/>
+    <col min="10" max="10" width="15.8984375" style="9" customWidth="1"/>
+    <col min="11" max="11" width="20.69921875" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>58</v>
       </c>
@@ -901,22 +953,22 @@
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
     </row>
-    <row r="3" spans="1:11" s="5" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="24" t="s">
+    <row r="3" spans="1:11" s="5" customFormat="1" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-    </row>
-    <row r="4" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+    </row>
+    <row r="4" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B4" s="7"/>
       <c r="C4" s="8"/>
       <c r="D4" s="8"/>
@@ -928,7 +980,7 @@
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
@@ -936,37 +988,39 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="21" t="s">
+      <c r="C6" s="26"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="H6" s="21" t="s">
+      <c r="H6" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="I6" s="21" t="s">
+      <c r="I6" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="J6" s="21" t="s">
+      <c r="J6" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="18" t="s">
+      <c r="K6" s="19" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="19"/>
+    <row r="7" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="20"/>
       <c r="B7" s="15" t="s">
         <v>36</v>
       </c>
@@ -976,17 +1030,15 @@
       <c r="D7" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="E7" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
-      <c r="K7" s="19"/>
-    </row>
-    <row r="8" spans="1:11" s="2" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E7" s="29"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="20"/>
+    </row>
+    <row r="8" spans="1:11" s="2" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="16" t="s">
         <v>40</v>
       </c>
@@ -1021,7 +1073,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
       <c r="E10" s="14"/>
@@ -1032,16 +1084,17 @@
       <c r="J10" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="K6:K7"/>
-    <mergeCell ref="B6:E6"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="F6:F7"/>
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="J6:J7"/>
     <mergeCell ref="H6:H7"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="E6:E7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>
@@ -1056,14 +1109,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.58203125" defaultRowHeight="21.9" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.08203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.1640625" customWidth="1"/>
-    <col min="3" max="3" width="100.58203125" customWidth="1"/>
+    <col min="1" max="1" width="5.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.19921875" customWidth="1"/>
+    <col min="3" max="3" width="100.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1074,7 +1127,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>1001</v>
       </c>
@@ -1085,7 +1138,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>1002</v>
       </c>
@@ -1096,7 +1149,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1004</v>
       </c>
@@ -1107,7 +1160,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>1005</v>
       </c>
@@ -1118,7 +1171,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>1006</v>
       </c>
@@ -1129,7 +1182,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>1007</v>
       </c>
@@ -1140,7 +1193,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>1017</v>
       </c>
@@ -1151,7 +1204,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>1018</v>
       </c>
@@ -1162,7 +1215,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>2003</v>
       </c>
@@ -1173,7 +1226,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>2005</v>
       </c>
@@ -1184,7 +1237,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>2008</v>
       </c>
@@ -1195,7 +1248,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>2009</v>
       </c>
@@ -1206,7 +1259,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>2011</v>
       </c>
@@ -1217,7 +1270,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>2014</v>
       </c>
@@ -1228,7 +1281,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>2016</v>
       </c>
@@ -1239,7 +1292,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>2018</v>
       </c>
@@ -1250,7 +1303,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>2022</v>
       </c>
@@ -1261,7 +1314,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>2025</v>
       </c>
@@ -1272,7 +1325,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>2032</v>
       </c>
@@ -1283,7 +1336,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>2034</v>
       </c>
@@ -1294,7 +1347,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>2037</v>
       </c>
@@ -1305,7 +1358,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>4010</v>
       </c>
@@ -1316,7 +1369,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>4017</v>
       </c>
@@ -1327,7 +1380,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>5006</v>
       </c>
@@ -1338,7 +1391,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>5007</v>
       </c>
@@ -1349,7 +1402,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>5011</v>
       </c>

</xml_diff>

<commit_message>
use state label placeholders
</commit_message>
<xml_diff>
--- a/api/templates/all_results/en.xlsx
+++ b/api/templates/all_results/en.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\all_results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\all_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F9EBA44-F8B5-46DF-9F2A-40A28D26D09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="815"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -136,12 +135,6 @@
     <t>&lt;stateName&gt;</t>
   </si>
   <si>
-    <t>State</t>
-  </si>
-  <si>
-    <t>LGA</t>
-  </si>
-  <si>
     <t>&lt;lgaName&gt;</t>
   </si>
   <si>
@@ -206,12 +199,18 @@
   </si>
   <si>
     <t>There are &lt;PerformanceTotalRecordLimit&gt; more records, but report size is limited to &lt;PerformanceQueryLimit&gt; records for performance reasons. If you need more results please filter them by any of the possible filters we are providing.</t>
+  </si>
+  <si>
+    <t>&lt;StateLabel&gt;</t>
+  </si>
+  <si>
+    <t>&lt;LgaLabel&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -579,7 +578,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -916,7 +915,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K10"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -940,7 +939,7 @@
     </row>
     <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8"/>
@@ -955,7 +954,7 @@
     </row>
     <row r="3" spans="1:11" s="5" customFormat="1" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="18" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B3" s="18"/>
       <c r="C3" s="18"/>
@@ -990,45 +989,45 @@
     </row>
     <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C6" s="26"/>
       <c r="D6" s="27"/>
       <c r="E6" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="H6" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="I6" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="J6" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="K6" s="19" t="s">
         <v>42</v>
-      </c>
-      <c r="F6" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="G6" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="H6" s="22" t="s">
-        <v>56</v>
-      </c>
-      <c r="I6" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="K6" s="19" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="20"/>
       <c r="B7" s="15" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E7" s="29"/>
       <c r="F7" s="23"/>
@@ -1040,37 +1039,37 @@
     </row>
     <row r="8" spans="1:11" s="2" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="16" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D8" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="F8" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="J8" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="K8" s="12" t="s">
         <v>43</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="I8" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="J8" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="K8" s="12" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
@@ -1107,7 +1106,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C27"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>

<commit_message>
Adding new fields to the Module Swaps report
</commit_message>
<xml_diff>
--- a/api/templates/all_results/en.xlsx
+++ b/api/templates/all_results/en.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26626"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\all_results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\all_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BDBE1EB-07D5-451E-82BD-E9CC96814096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="815"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -210,7 +211,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -419,7 +420,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -437,51 +438,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="43" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -491,21 +462,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="Bad" xfId="43" builtinId="27"/>
@@ -578,7 +549,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -915,172 +886,176 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K10"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.5" style="5" customWidth="1"/>
-    <col min="2" max="2" width="23.09765625" style="7" customWidth="1"/>
-    <col min="3" max="3" width="22.3984375" style="8" customWidth="1"/>
-    <col min="4" max="4" width="18.5" style="8" customWidth="1"/>
-    <col min="5" max="5" width="28.59765625" style="9" customWidth="1"/>
-    <col min="6" max="6" width="21.3984375" style="9" customWidth="1"/>
-    <col min="7" max="7" width="21.296875" style="9" customWidth="1"/>
-    <col min="8" max="8" width="11.8984375" style="9" customWidth="1"/>
-    <col min="9" max="9" width="17.19921875" style="9" customWidth="1"/>
-    <col min="10" max="10" width="15.8984375" style="9" customWidth="1"/>
-    <col min="11" max="11" width="20.69921875" style="9" customWidth="1"/>
+    <col min="1" max="1" width="22.5" style="20" customWidth="1"/>
+    <col min="2" max="2" width="23.09765625" style="20" customWidth="1"/>
+    <col min="3" max="3" width="22.3984375" style="20" customWidth="1"/>
+    <col min="4" max="4" width="18.5" style="20" customWidth="1"/>
+    <col min="5" max="5" width="28.59765625" style="20" customWidth="1"/>
+    <col min="6" max="6" width="21.3984375" style="20" customWidth="1"/>
+    <col min="7" max="7" width="21.296875" style="20" customWidth="1"/>
+    <col min="8" max="8" width="11.8984375" style="20" customWidth="1"/>
+    <col min="9" max="9" width="17.19921875" style="20" customWidth="1"/>
+    <col min="10" max="10" width="15.8984375" style="20" customWidth="1"/>
+    <col min="11" max="11" width="20.69921875" style="20" customWidth="1"/>
+    <col min="12" max="16384" width="11" style="20"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" customFormat="1" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
         <v>34</v>
       </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
     </row>
     <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
     </row>
     <row r="3" spans="1:11" s="5" customFormat="1" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
     </row>
     <row r="4" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="7"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+    </row>
+    <row r="6" spans="1:11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="26"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="28" t="s">
+      <c r="C6" s="16"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="22" t="s">
+      <c r="G6" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="H6" s="22" t="s">
+      <c r="H6" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="I6" s="22" t="s">
+      <c r="I6" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="J6" s="22" t="s">
+      <c r="J6" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="K6" s="19" t="s">
+      <c r="K6" s="10" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="20"/>
-      <c r="B7" s="15" t="s">
+      <c r="A7" s="11"/>
+      <c r="B7" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="29"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="24"/>
-      <c r="K7" s="20"/>
-    </row>
-    <row r="8" spans="1:11" s="2" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="16" t="s">
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="11"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I8" s="17" t="s">
+      <c r="I8" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="J8" s="17" t="s">
+      <c r="J8" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="K8" s="12" t="s">
+      <c r="K8" s="18" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -1106,7 +1081,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C27"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>

<commit_message>
Changed the header color of the all results report
</commit_message>
<xml_diff>
--- a/api/templates/all_results/en.xlsx
+++ b/api/templates/all_results/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\all_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BDBE1EB-07D5-451E-82BD-E9CC96814096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{883DD76E-8312-4124-91E7-C2636DB78129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -277,13 +277,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor rgb="FF3CC0DD"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -418,9 +418,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -441,42 +441,41 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="43" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="43" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="Bad" xfId="43" builtinId="27"/>
@@ -554,6 +553,11 @@
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="FF3CC0DD"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -890,21 +894,20 @@
   <dimension ref="A1:K10"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.5" style="20" customWidth="1"/>
-    <col min="2" max="2" width="23.09765625" style="20" customWidth="1"/>
-    <col min="3" max="3" width="22.3984375" style="20" customWidth="1"/>
-    <col min="4" max="4" width="18.5" style="20" customWidth="1"/>
-    <col min="5" max="5" width="28.59765625" style="20" customWidth="1"/>
-    <col min="6" max="6" width="21.3984375" style="20" customWidth="1"/>
-    <col min="7" max="7" width="21.296875" style="20" customWidth="1"/>
-    <col min="8" max="8" width="11.8984375" style="20" customWidth="1"/>
-    <col min="9" max="9" width="17.19921875" style="20" customWidth="1"/>
-    <col min="10" max="10" width="15.8984375" style="20" customWidth="1"/>
-    <col min="11" max="11" width="20.69921875" style="20" customWidth="1"/>
-    <col min="12" max="16384" width="11" style="20"/>
+    <col min="1" max="1" width="22.5" customWidth="1"/>
+    <col min="2" max="2" width="23.09765625" customWidth="1"/>
+    <col min="3" max="3" width="22.3984375" customWidth="1"/>
+    <col min="4" max="4" width="18.5" customWidth="1"/>
+    <col min="5" max="5" width="28.59765625" customWidth="1"/>
+    <col min="6" max="6" width="21.3984375" customWidth="1"/>
+    <col min="7" max="7" width="21.296875" customWidth="1"/>
+    <col min="8" max="8" width="11.8984375" customWidth="1"/>
+    <col min="9" max="9" width="17.19921875" customWidth="1"/>
+    <col min="10" max="10" width="15.8984375" customWidth="1"/>
+    <col min="11" max="11" width="20.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
         <v>34</v>
       </c>
@@ -927,25 +930,25 @@
       <c r="D2" s="7"/>
     </row>
     <row r="3" spans="1:11" s="5" customFormat="1" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
     </row>
     <row r="4" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
     </row>
-    <row r="5" spans="1:11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
@@ -962,100 +965,100 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="12" t="s">
+      <c r="C6" s="14"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F6" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="G6" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="H6" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="I6" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="J6" s="12" t="s">
+      <c r="J6" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="K6" s="10" t="s">
+      <c r="K6" s="12" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="11"/>
-      <c r="B7" s="8" t="s">
+      <c r="A7" s="17"/>
+      <c r="B7" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="14"/>
-      <c r="K7" s="11"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
+      <c r="K7" s="17"/>
     </row>
     <row r="8" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="I8" s="18" t="s">
+      <c r="I8" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="J8" s="18" t="s">
+      <c r="J8" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="K8" s="18" t="s">
+      <c r="K8" s="8" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
Freeze header row in all results xlsx template
</commit_message>
<xml_diff>
--- a/api/templates/all_results/en.xlsx
+++ b/api/templates/all_results/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26827"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\all_results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\all_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{883DD76E-8312-4124-91E7-C2636DB78129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AFA15A0-ADD2-4665-B911-EF883C892C43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11835" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -446,12 +446,27 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="43" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -459,21 +474,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -892,22 +892,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K10"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.5" customWidth="1"/>
-    <col min="2" max="2" width="23.09765625" customWidth="1"/>
-    <col min="3" max="3" width="22.3984375" customWidth="1"/>
+    <col min="2" max="2" width="23.125" customWidth="1"/>
+    <col min="3" max="3" width="22.375" customWidth="1"/>
     <col min="4" max="4" width="18.5" customWidth="1"/>
-    <col min="5" max="5" width="28.59765625" customWidth="1"/>
-    <col min="6" max="6" width="21.3984375" customWidth="1"/>
-    <col min="7" max="7" width="21.296875" customWidth="1"/>
-    <col min="8" max="8" width="11.8984375" customWidth="1"/>
-    <col min="9" max="9" width="17.19921875" customWidth="1"/>
-    <col min="10" max="10" width="15.8984375" customWidth="1"/>
-    <col min="11" max="11" width="20.69921875" customWidth="1"/>
+    <col min="5" max="5" width="28.625" customWidth="1"/>
+    <col min="6" max="6" width="23.5" customWidth="1"/>
+    <col min="7" max="7" width="21.25" customWidth="1"/>
+    <col min="8" max="8" width="11.875" customWidth="1"/>
+    <col min="9" max="9" width="17.25" customWidth="1"/>
+    <col min="10" max="10" width="15.875" customWidth="1"/>
+    <col min="11" max="11" width="20.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>34</v>
       </c>
@@ -922,33 +922,33 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
     </row>
-    <row r="3" spans="1:11" s="5" customFormat="1" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
+    <row r="3" spans="1:11" s="5" customFormat="1" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-    </row>
-    <row r="4" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+    </row>
+    <row r="4" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
@@ -965,57 +965,57 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
+    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16" t="s">
+      <c r="C6" s="19"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="G6" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="H6" s="16" t="s">
+      <c r="H6" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="I6" s="16" t="s">
+      <c r="I6" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="J6" s="16" t="s">
+      <c r="J6" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="K6" s="12" t="s">
+      <c r="K6" s="13" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="17"/>
-      <c r="B7" s="18" t="s">
+    <row r="7" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="14"/>
+      <c r="B7" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="20"/>
-      <c r="I7" s="20"/>
-      <c r="J7" s="20"/>
-      <c r="K7" s="17"/>
-    </row>
-    <row r="8" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="14"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>38</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>
@@ -1086,14 +1086,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.09765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.19921875" customWidth="1"/>
-    <col min="3" max="3" width="100.59765625" customWidth="1"/>
+    <col min="1" max="1" width="5.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.25" customWidth="1"/>
+    <col min="3" max="3" width="100.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1104,7 +1104,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1001</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1002</v>
       </c>
@@ -1126,7 +1126,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>1004</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>1005</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>1006</v>
       </c>
@@ -1159,7 +1159,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>1007</v>
       </c>
@@ -1170,7 +1170,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>1017</v>
       </c>
@@ -1181,7 +1181,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>1018</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>2003</v>
       </c>
@@ -1203,7 +1203,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>2005</v>
       </c>
@@ -1214,7 +1214,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>2008</v>
       </c>
@@ -1225,7 +1225,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>2009</v>
       </c>
@@ -1236,7 +1236,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>2011</v>
       </c>
@@ -1247,7 +1247,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>2014</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>2016</v>
       </c>
@@ -1269,7 +1269,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>2018</v>
       </c>
@@ -1280,7 +1280,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>2022</v>
       </c>
@@ -1291,7 +1291,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>2025</v>
       </c>
@@ -1302,7 +1302,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>2032</v>
       </c>
@@ -1313,7 +1313,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>2034</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>2037</v>
       </c>
@@ -1335,7 +1335,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>4010</v>
       </c>
@@ -1346,7 +1346,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>4017</v>
       </c>
@@ -1357,7 +1357,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>5006</v>
       </c>
@@ -1368,7 +1368,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>5007</v>
       </c>
@@ -1379,7 +1379,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>5011</v>
       </c>

</xml_diff>

<commit_message>
[feat/ASP-7746-Device-and-Sites-Summary-Report-include-Total-line] Updated all results template
</commit_message>
<xml_diff>
--- a/api/templates/all_results/en.xlsx
+++ b/api/templates/all_results/en.xlsx
@@ -1,23 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10420"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\all_results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/all_results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AFA15A0-ADD2-4665-B911-EF883C892C43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314E0DEE-407C-4F42-A346-1A02542489AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11835" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="20520" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
     <sheet name="Error Codes" sheetId="3" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
     </ext>
@@ -441,40 +452,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="43" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="43" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="44">
@@ -891,23 +902,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K10"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.5" customWidth="1"/>
-    <col min="2" max="2" width="23.125" customWidth="1"/>
-    <col min="3" max="3" width="22.375" customWidth="1"/>
+    <col min="2" max="2" width="23.1640625" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" customWidth="1"/>
     <col min="4" max="4" width="18.5" customWidth="1"/>
-    <col min="5" max="5" width="28.625" customWidth="1"/>
+    <col min="5" max="5" width="28.6640625" customWidth="1"/>
     <col min="6" max="6" width="23.5" customWidth="1"/>
-    <col min="7" max="7" width="21.25" customWidth="1"/>
-    <col min="8" max="8" width="11.875" customWidth="1"/>
-    <col min="9" max="9" width="17.25" customWidth="1"/>
-    <col min="10" max="10" width="15.875" customWidth="1"/>
-    <col min="11" max="11" width="20.75" customWidth="1"/>
+    <col min="7" max="7" width="21.1640625" customWidth="1"/>
+    <col min="8" max="8" width="11.83203125" customWidth="1"/>
+    <col min="9" max="9" width="17.1640625" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" customWidth="1"/>
+    <col min="11" max="11" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>34</v>
       </c>
@@ -922,33 +933,33 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
     </row>
-    <row r="3" spans="1:11" s="5" customFormat="1" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:11" s="5" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-    </row>
-    <row r="4" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+    </row>
+    <row r="4" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
@@ -965,100 +976,100 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="19"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="15" t="s">
+      <c r="C6" s="17"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="H6" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="I6" s="15" t="s">
+      <c r="I6" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="J6" s="15" t="s">
+      <c r="J6" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="K6" s="13" t="s">
+      <c r="K6" s="11" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="14"/>
-      <c r="B7" s="11" t="s">
+    <row r="7" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="12"/>
+      <c r="B7" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="14"/>
-    </row>
-    <row r="8" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="12"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="K8" s="19" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -1086,14 +1097,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="22" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.25" customWidth="1"/>
-    <col min="3" max="3" width="100.625" customWidth="1"/>
+    <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.1640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1104,7 +1115,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>1001</v>
       </c>
@@ -1115,7 +1126,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1002</v>
       </c>
@@ -1126,7 +1137,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>1004</v>
       </c>
@@ -1137,7 +1148,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>1005</v>
       </c>
@@ -1148,7 +1159,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>1006</v>
       </c>
@@ -1159,7 +1170,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>1007</v>
       </c>
@@ -1170,7 +1181,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>1017</v>
       </c>
@@ -1181,7 +1192,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>1018</v>
       </c>
@@ -1192,7 +1203,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>2003</v>
       </c>
@@ -1203,7 +1214,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>2005</v>
       </c>
@@ -1214,7 +1225,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>2008</v>
       </c>
@@ -1225,7 +1236,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>2009</v>
       </c>
@@ -1236,7 +1247,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>2011</v>
       </c>
@@ -1247,7 +1258,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>2014</v>
       </c>
@@ -1258,7 +1269,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>2016</v>
       </c>
@@ -1269,7 +1280,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>2018</v>
       </c>
@@ -1280,7 +1291,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>2022</v>
       </c>
@@ -1291,7 +1302,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>2025</v>
       </c>
@@ -1302,7 +1313,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>2032</v>
       </c>
@@ -1313,7 +1324,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>2034</v>
       </c>
@@ -1324,7 +1335,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>2037</v>
       </c>
@@ -1335,7 +1346,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>4010</v>
       </c>
@@ -1346,7 +1357,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>4017</v>
       </c>
@@ -1357,7 +1368,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>5006</v>
       </c>
@@ -1368,7 +1379,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
         <v>5007</v>
       </c>
@@ -1379,7 +1390,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>5011</v>
       </c>

</xml_diff>

<commit_message>
[feat/ASP-7746-Device-and-Sites-Summary-Report-include-Total-line] Finished totals rows when avoid streaming
</commit_message>
<xml_diff>
--- a/api/templates/all_results/en.xlsx
+++ b/api/templates/all_results/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/all_results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314E0DEE-407C-4F42-A346-1A02542489AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24775B0C-C12E-2541-8551-E404C13E62C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="20520" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -223,7 +223,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -259,14 +259,6 @@
       <u/>
       <sz val="12"/>
       <color theme="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -429,9 +421,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -452,40 +444,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="43" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="43" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="44">
@@ -902,7 +893,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.5" customWidth="1"/>
@@ -941,19 +932,19 @@
       <c r="D2" s="7"/>
     </row>
     <row r="3" spans="1:11" s="5" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
     </row>
     <row r="4" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C4" s="7"/>
@@ -977,99 +968,89 @@
       <c r="K5" s="2"/>
     </row>
     <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="17"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="13" t="s">
+      <c r="C6" s="18"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="I6" s="13" t="s">
+      <c r="I6" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="J6" s="13" t="s">
+      <c r="J6" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="K6" s="12" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="12"/>
-      <c r="B7" s="9" t="s">
+      <c r="A7" s="13"/>
+      <c r="B7" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="12"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="13"/>
     </row>
     <row r="8" spans="1:11" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="20" t="s">
+      <c r="H8" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="I8" s="19" t="s">
+      <c r="I8" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="J8" s="19" t="s">
+      <c r="J8" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="K8" s="19" t="s">
+      <c r="K8" s="9" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
[feat/ASP-8019-report-parameters] Fixed download report with cleared parameters issue
</commit_message>
<xml_diff>
--- a/api/templates/all_results/en.xlsx
+++ b/api/templates/all_results/en.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10531"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E7064EA-C3DD-A04E-8B93-B43B11177170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Results" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Error Codes" state="visible" r:id="rId5"/>
+    <sheet name="Results" sheetId="1" r:id="rId1"/>
+    <sheet name="Error Codes" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -197,43 +198,44 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="16"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="16"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="4">
@@ -263,38 +265,64 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -308,28 +336,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -339,6 +349,27 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -614,9 +645,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="11" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.5" customWidth="1"/>
     <col min="2" max="2" width="23.1640625" customWidth="1"/>
@@ -630,7 +661,7 @@
     <col min="10" max="10" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -644,39 +675,37 @@
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
     </row>
-    <row r="2" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
     </row>
-    <row r="3" ht="29" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" ht="29" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:10" s="2" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-    </row>
-    <row r="5" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
+    </row>
+    <row r="5" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -692,81 +721,81 @@
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
     </row>
-    <row r="7" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="8" t="s">
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" ht="31.5" customHeight="1" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
-      <c r="B8" s="6" t="s">
+    <row r="8" spans="1:10" s="6" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="14"/>
+      <c r="B8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="10"/>
-    </row>
-    <row r="9" ht="15.5" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="14"/>
+    </row>
+    <row r="9" spans="1:10" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="I9" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="J9" s="7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -783,319 +812,319 @@
     <mergeCell ref="J7:J8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967292" verticalDpi="4294967292"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.6640625" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="22" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" customWidth="1"/>
     <col min="2" max="2" width="39.1640625" customWidth="1"/>
     <col min="3" max="3" width="100.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="16">
+    <row r="2" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="10">
         <v>1001</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="10" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="16">
+    <row r="3" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="10">
         <v>1002</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="16">
+    <row r="4" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="10">
         <v>1004</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="16">
+    <row r="5" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="10">
         <v>1005</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="10" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="16">
+    <row r="6" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="10">
         <v>1006</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="16">
+    <row r="7" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="10">
         <v>1007</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="10" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="16">
+    <row r="8" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="10">
         <v>1017</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="10" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="16">
+    <row r="9" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="10">
         <v>1018</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="16">
+    <row r="10" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="10">
         <v>2003</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="10" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="16">
+    <row r="11" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="10">
         <v>2005</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="16">
+    <row r="12" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="10">
         <v>2008</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="16">
+    <row r="13" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="10">
         <v>2009</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="10" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="16">
+    <row r="14" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="10">
         <v>2011</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="16">
+    <row r="15" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="10">
         <v>2014</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="10" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="16">
+    <row r="16" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="10">
         <v>2016</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="16">
+    <row r="17" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="10">
         <v>2018</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="10" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="16">
+    <row r="18" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="10">
         <v>2022</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="10" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="16">
+    <row r="19" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="10">
         <v>2025</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="C19" s="10" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="16">
+    <row r="20" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="10">
         <v>2032</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="10" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="16">
+    <row r="21" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="10">
         <v>2034</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="16">
+    <row r="22" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="10">
         <v>2037</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="16" t="s">
+      <c r="C22" s="10" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="16">
+    <row r="23" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="10">
         <v>4010</v>
       </c>
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="16" t="s">
+      <c r="C23" s="10" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="16">
+    <row r="24" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="10">
         <v>4017</v>
       </c>
-      <c r="B24" s="16" t="s">
+      <c r="B24" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="10" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="16">
+    <row r="25" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="10">
         <v>5006</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C25" s="16" t="s">
+      <c r="C25" s="10" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="16">
+    <row r="26" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="10">
         <v>5007</v>
       </c>
-      <c r="B26" s="16" t="s">
+      <c r="B26" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="16" t="s">
+      <c r="C26" s="10" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="27" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="16">
+    <row r="27" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="10">
         <v>5011</v>
       </c>
-      <c r="B27" s="16" t="s">
+      <c r="B27" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C27" s="10" t="s">
         <v>58</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>